<commit_message>
Inspector import: AvailabilityDate is a dateTime, use ISO 8601 text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/09-airlite-product-template/Airlite_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/09-airlite-product-template/Airlite_RCA_Import_Inspector.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Fill yellow cells. Product_Owner__c needs the owner's User Id (Data Export: SELECT Id FROM User WHERE Email = '...'). AvailabilityDate as YYYY-MM-DD. BasedOn links the product to the classification so it inherits the attributes.</t>
+          <t>Fill yellow cells. Product_Owner__c needs the owner's User Id (Data Export: SELECT Id FROM User WHERE Email = '...'). AvailabilityDate is a date/time field: enter it as text, e.g. 2026-01-01T00:00:00.000Z (type a leading apostrophe in Excel so it is not reformatted to 01/01/2026). BasedOn links the product to the classification so it inherits the attributes.</t>
         </is>
       </c>
     </row>
@@ -7895,7 +7895,7 @@
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="36" customWidth="1" min="12" max="12"/>
   </cols>
@@ -8006,7 +8006,7 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>&lt;YYYY-MM-DD&gt;</t>
+          <t>&lt;YYYY-MM-DDT00:00:00.000Z&gt;</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Inspector import: prefix AttributeDefinition Name to keep it org-unique
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/09-airlite-product-template/Airlite_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/09-airlite-product-template/Airlite_RCA_Import_Inspector.xlsx
@@ -513,7 +513,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Includes the 12 calculated output attributes (Description starts 'Calculated').</t>
+          <t>Name is prefixed 'AIR ' because AttributeDefinition Name must be unique across the org; Label (shown to users) is unchanged. Includes the 12 calculated output attributes (Description starts 'Calculated').</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1445,7 @@
   <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -1518,7 +1518,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>AIR Version</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1575,7 +1575,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Width</t>
+          <t>AIR Width</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1624,7 +1624,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Length</t>
+          <t>AIR Length</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1677,7 +1677,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Flange Width</t>
+          <t>AIR Flange Width</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1726,7 +1726,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Flange Length</t>
+          <t>AIR Flange Length</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1775,7 +1775,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Insulation</t>
+          <t>AIR Insulation</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1832,7 +1832,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Louvre</t>
+          <t>AIR Louvre</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1885,7 +1885,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Controls</t>
+          <t>AIR Controls</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1938,7 +1938,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Thermal Release</t>
+          <t>AIR Thermal Release</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1995,7 +1995,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Control Bracket Design</t>
+          <t>AIR Control Bracket Design</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2048,7 +2048,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Base Design</t>
+          <t>AIR Base Design</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2101,7 +2101,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Flange Type</t>
+          <t>AIR Flange Type</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2158,7 +2158,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Coating</t>
+          <t>AIR Coating</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2215,7 +2215,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>RAL Colour</t>
+          <t>AIR RAL Colour</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Coating Thickness</t>
+          <t>AIR Coating Thickness</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2321,7 +2321,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Installation Type</t>
+          <t>AIR Installation Type</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -2374,7 +2374,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Mounting Angle</t>
+          <t>AIR Mounting Angle</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2423,7 +2423,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Wind Baffle</t>
+          <t>AIR Wind Baffle</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -2476,7 +2476,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>AIR Delivery</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -2533,7 +2533,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Snow Load</t>
+          <t>AIR Snow Load</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -2582,7 +2582,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Wind Load</t>
+          <t>AIR Wind Load</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -2631,7 +2631,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Ambient Air Temperature</t>
+          <t>AIR Ambient Air Temperature</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -2688,7 +2688,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Pressure Day to Day</t>
+          <t>AIR Pressure Day to Day</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -2741,7 +2741,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Pressure Smoke Ventilation</t>
+          <t>AIR Pressure Smoke Ventilation</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -2794,7 +2794,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Cylinder</t>
+          <t>AIR Cylinder</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -2843,7 +2843,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>CO2 Bottle</t>
+          <t>AIR CO2 Bottle</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -2892,7 +2892,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Pressure Standby Reservoir</t>
+          <t>AIR Pressure Standby Reservoir</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -2941,7 +2941,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Electric Drive</t>
+          <t>AIR Electric Drive</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -2990,7 +2990,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Wind Suction Load WL</t>
+          <t>AIR Wind Suction Load WL</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -3039,7 +3039,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Geometric Area Av</t>
+          <t>AIR Geometric Area Av</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -3088,7 +3088,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Aerodynamic Area Aa</t>
+          <t>AIR Aerodynamic Area Aa</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>U-Value</t>
+          <t>AIR U-Value</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -3186,7 +3186,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Louvre Weight</t>
+          <t>AIR Louvre Weight</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -3235,7 +3235,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Total Weight</t>
+          <t>AIR Total Weight</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -3284,7 +3284,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Max SL Pneumatic Cylinder</t>
+          <t>AIR Max SL Pneumatic Cylinder</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -3333,7 +3333,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Max SL Motor</t>
+          <t>AIR Max SL Motor</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Skill: make AttributeDefinition Name and picklist value Code org-unique by default
- generate_import_csvs.py prefixes AttributeDefinition.Name (<PREFIX> <Name>) and
  AttributePicklistValue.Code (<PREFIX>_<Picklist>_<Value>); --legacy reproduces ECO.
- Add build_inspector_import.py (Salesforce Inspector Reloaded workbook) to the skill.
- Document the rule and the Inspector import lessons (dateTime, owner Id, lookups).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/09-airlite-product-template/Airlite_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/09-airlite-product-template/Airlite_RCA_Import_Inspector.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Several categories may already exist from ECO (Device_Configuration, Filling, Control_and_Drive, Base_and_Flange, Options, Finish, Calculated_Outputs). A DUPLICATE_VALUE error on those rows is fine – they are reused.</t>
+          <t>Several categories may already exist from earlier products, e.g. ECO (Device_Configuration, Filling, Control_and_Drive, Base_and_Flange, Options, Finish, Calculated_Outputs). A DUPLICATE_VALUE error on those rows is fine – they are reused.</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Fill yellow cells. Product_Owner__c needs the owner's User Id (Data Export: SELECT Id FROM User WHERE Email = '...'). AvailabilityDate is a date/time field: enter it as text, e.g. 2026-01-01T00:00:00.000Z (type a leading apostrophe in Excel so it is not reformatted to 01/01/2026). BasedOn links the product to the classification so it inherits the attributes.</t>
+          <t>Fill yellow cells. Product_Owner__c needs the owner's User Id starting 005, not an alias or e-mail (Data Export: SELECT Id FROM User WHERE Email = '...'). AvailabilityDate is a date/time field: enter it as text, e.g. 2026-01-01T00:00:00.000Z (type a leading apostrophe in Excel so it is not reformatted to 01/01/2026). BasedOn links the product to the classification so it inherits the attributes.</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ProductId = the Id Inspector returns in step 06. ProductCategoryId: Data Export SELECT Id, Name FROM ProductCategory WHERE Name = 'Natural Ventilation'.</t>
+          <t>ProductId = the Id Inspector returns in step 06. ProductCategoryId: Data Export SELECT Id, Name FROM ProductCategory WHERE Name = '&lt;category from the Product sheet&gt;'.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -747,7 +747,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>&lt;Id of Natural Ventilation&gt;</t>
+          <t>&lt;ProductCategory Id&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Skill: give the Data Export query for every Id needed during import
Per-step SOQL (owner User Id, product family, Product2 Id, ProductCategory Id
with catalog, Pricebook2 Id, attribute check) in the reference doc, SKILL.md
and the Import Steps tab of the Inspector workbook. Fix the tab 06 note that
told users to type an apostrophe before the dateTime value.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/09-airlite-product-template/Airlite_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/09-airlite-product-template/Airlite_RCA_Import_Inspector.xlsx
@@ -450,13 +450,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="110" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,6 +481,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Data Export query to find the Ids for this step</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -496,6 +502,7 @@
         <v>15</v>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -516,6 +523,7 @@
           <t>Name is prefixed 'AIR ' because AttributeDefinition Name must be unique across the org; Label (shown to users) is unchanged. Includes the 12 calculated output attributes (Description starts 'Calculated').</t>
         </is>
       </c>
+      <c r="E3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -536,6 +544,7 @@
           <t>Code is prefixed (AIR_&lt;Picklist&gt;_&lt;Value&gt;) so it can't clash with ECO codes already in the org; Value is unchanged.</t>
         </is>
       </c>
+      <c r="E4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -556,6 +565,7 @@
           <t>Several categories may already exist from earlier products, e.g. ECO (Device_Configuration, Filling, Control_and_Drive, Base_and_Flange, Options, Finish, Calculated_Outputs). A DUPLICATE_VALUE error on those rows is fine – they are reused.</t>
         </is>
       </c>
+      <c r="E5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -572,6 +582,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -589,7 +600,15 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Fill yellow cells. Product_Owner__c needs the owner's User Id starting 005, not an alias or e-mail (Data Export: SELECT Id FROM User WHERE Email = '...'). AvailabilityDate is a date/time field: enter it as text, e.g. 2026-01-01T00:00:00.000Z (type a leading apostrophe in Excel so it is not reformatted to 01/01/2026). BasedOn links the product to the classification so it inherits the attributes.</t>
+          <t>Fill yellow cells. Product_Owner__c = owner's User Id (starts 005, not alias/e-mail). AvailabilityDate is a date/time: type 2026-01-01T00:00:00.000Z exactly, NO apostrophe (cells are Text). Product_Family_ROD__c optional – use an existing value. BasedOn links the product to the classification so it inherits the attributes.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Product owner User Id (005…):
+SELECT Id, Name, Alias, Email FROM User WHERE Alias = '&lt;alias&gt;' OR Email = '&lt;e-mail&gt;'
+Existing product family values:
+SELECT Product_Family_ROD__c, COUNT(Id) FROM Product2 WHERE Product_Family_ROD__c != null GROUP BY Product_Family_ROD__c</t>
         </is>
       </c>
     </row>
@@ -608,6 +627,12 @@
         <v>36</v>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Check all attributes from step 02 exist:
+SELECT Code, Name, DataType FROM AttributeDefinition WHERE Code LIKE 'AIR_%' ORDER BY Code</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -628,6 +653,7 @@
           <t>Calculated outputs are IsReadOnly = true. DisplayType is only set (Dropdown) for picklists.</t>
         </is>
       </c>
+      <c r="E9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -645,7 +671,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ProductId = the Id Inspector returns in step 06. ProductCategoryId: Data Export SELECT Id, Name FROM ProductCategory WHERE Name = '&lt;category from the Product sheet&gt;'.</t>
+          <t>Object = ProductCategoryProduct (Inspector keeps the last object selected – change it!). Both columns need record Ids (01t… / 0ZG…), not names – see the Data Export queries on the Import Steps tab.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>ProductId (01t…) – the product from step 06:
+SELECT Id, Name, ProductCode FROM Product2 WHERE ProductCode = 'AIR'
+ProductCategoryId (0ZG…) with its catalog:
+SELECT Id, Name, Catalog.Name, CatalogId FROM ProductCategory WHERE Name LIKE '%&lt;category&gt;%' ORDER BY Catalog.Name, Name
+Which category/catalog a similar product uses:
+SELECT ProductCategoryId, ProductCategory.Name, ProductCategory.Catalog.Name FROM ProductCategoryProduct WHERE Product.ProductCode = '&lt;similar product code&gt;'</t>
         </is>
       </c>
     </row>
@@ -668,6 +704,12 @@
           <t>Skip until the factory supplies prices. Standard Price Book entry first, then the KLAW price book.</t>
         </is>
       </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Pricebook2Id:
+SELECT Id, Name, IsStandard FROM Pricebook2 WHERE IsActive = true</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -688,12 +730,14 @@
           <t>Skip until prices are known (see the template's Configurable Product Pricing tab).</t>
         </is>
       </c>
+      <c r="E12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="2" t="n"/>
       <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -708,6 +752,7 @@
       </c>
       <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>